<commit_message>
added export of radaplot
</commit_message>
<xml_diff>
--- a/tables_and_figures/table1_symptomes_per_questionnaire.xlsx
+++ b/tables_and_figures/table1_symptomes_per_questionnaire.xlsx
@@ -436,33 +436,33 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PRAQ</t>
+          <t>SAQLI</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C2" t="n">
         <v>6</v>
       </c>
       <c r="D2" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SAQLI</t>
+          <t>OSAPOSI</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C3" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D3" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4">
@@ -484,39 +484,39 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>OSAPOSI</t>
+          <t>MOSAS</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>STAMP</t>
+          <t>PRAQ</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D6" t="n">
-        <v>12</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>MOSAS</t>
+          <t>STAMP</t>
         </is>
       </c>
       <c r="B7" t="n">

</xml_diff>